<commit_message>
data(gold): corrected frozen gold set; steps as integers in the output
The workbook (sha256 e4214ccd..., pinned) moves the 11 shifted rows (A25-A28,
A30, A37, A44, B37, B42, C7, C8) back into their columns, with 11 Changelog
entries; a cell-by-cell comparison shows no other change. No row has an
empty quote now. The jsonl output holds step as an integer (28 conversions,
logged in gold_manifest.json); the workbook keeps what was typed.
</commit_message>
<xml_diff>
--- a/data/gold/gold_set_annotations_final.xlsx
+++ b/data/gold/gold_set_annotations_final.xlsx
@@ -2159,27 +2159,27 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>mark</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>plots</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>Mark plots of 2.5m breadth with channels 30cm wide all around the seedbeds.</t>
         </is>
@@ -2212,27 +2212,27 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>seedbed length</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>8-10</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="S27" t="inlineStr">
         <is>
           <t>Length of the seed bed may vary from 8 to 10m according to soil and slope of the land.</t>
         </is>
@@ -2265,17 +2265,17 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>level</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>seedbed surface</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="S28" t="inlineStr">
         <is>
           <t>Level the surface of the seedbed, so that the water drains into the channel.</t>
         </is>
@@ -2308,22 +2308,22 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>sow</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>sprouted seeds</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>thin film of water</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>Sow the sprouted seeds uniformly on the seedbed having thin film of water in the surface.</t>
         </is>
@@ -2409,17 +2409,17 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>avoid</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>stagnation of water</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="S31" t="inlineStr">
         <is>
           <t>Care must be taken to avoid stagnation of water on the seedbed.</t>
         </is>
@@ -2850,32 +2850,32 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>apply</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>FYM or compost</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>tonne</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t>20 cents nursery</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="S38" t="inlineStr">
         <is>
           <t>Apply 1 tonne of fully decomposed FYM or compost to 20 cents nursery and spread the manure uniformly on dry soil.</t>
         </is>
@@ -3346,32 +3346,32 @@
           <t>rice</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>apply</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>ZnSO4</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="P45" t="inlineStr">
         <is>
           <t>cent</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
+      <c r="S45" t="inlineStr">
         <is>
           <t>Soil application of 100 g ZnSO4 /cent can be followed.</t>
         </is>
@@ -5642,12 +5642,12 @@
           <t>close planting</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>especially in BPH and leaffolder prone areas/seasons</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="S30" t="inlineStr">
         <is>
           <t>Avoid close planting, especially in BPH and leaffolder prone areas/seasons</t>
         </is>
@@ -5965,12 +5965,12 @@
           <t>synthetic pyrethroids</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="R36" t="inlineStr">
         <is>
           <t>Repeated application can cause resurgence of insect pests</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>Repeated application of the following insecticides can cause resurgence of insect pests Avoid spraying of synthetic pyrethroids and the following insecticides</t>
         </is>
@@ -6479,12 +6479,12 @@
           <t>golden yellow colour</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>moisture: 20%</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>When 90 % of the panicle are in golden yello w colour with the moisture content of 20% for short and medium duration varieties and 17% moisture for long duration varieties.</t>
         </is>
@@ -6547,12 +6547,12 @@
           <t>golden yellow colour</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>moisture: 17%</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>When 90 % of the panicle are in golden yello w colour with the moisture content of 20% for short and medium duration varieties and 17% moisture for long duration varieties.</t>
         </is>
@@ -7318,7 +7318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7377,7 +7377,6 @@
           <t>alternative</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>preferred</t>
@@ -7634,7 +7633,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -7694,7 +7692,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -7717,7 +7714,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -7750,7 +7746,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -7773,7 +7768,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -7806,7 +7800,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -7829,7 +7822,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -7862,7 +7854,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -7885,7 +7876,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -7918,7 +7908,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -7941,7 +7930,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8070,7 +8058,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -8093,7 +8080,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8222,7 +8208,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -8245,7 +8230,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8374,7 +8358,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -8397,7 +8380,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8526,7 +8508,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -8549,7 +8530,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8678,7 +8658,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -8701,7 +8680,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8830,7 +8808,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -8853,7 +8830,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -8982,7 +8958,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9005,7 +8980,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -9134,7 +9108,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9157,7 +9130,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -9286,7 +9258,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9309,7 +9280,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -9438,7 +9408,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9461,7 +9430,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -9590,7 +9558,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9613,7 +9580,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -9742,7 +9708,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9765,7 +9730,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -9926,7 +9890,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -9949,7 +9912,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10110,7 +10072,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10133,7 +10094,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10262,7 +10222,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10285,7 +10244,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10414,7 +10372,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10437,7 +10394,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10566,7 +10522,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10589,7 +10544,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10718,7 +10672,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10741,7 +10694,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10870,7 +10822,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10930,7 +10881,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -10953,7 +10903,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -10986,7 +10935,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -11009,7 +10957,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -11042,7 +10989,6 @@
           <t>general;</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -11065,7 +11011,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
           <t>general;</t>
@@ -11098,7 +11043,6 @@
           <t>BPH;</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>pest marker belongs in condition</t>
@@ -11121,7 +11065,6 @@
           <t>condition</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>BPH;</t>
@@ -11197,10 +11140,362 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>A25</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Frozen gold set: built from v3 by mechanical fixes only. No value, unit, basis or quote content was changed apart from removing the shared list intro from B quotes. Remaining disagreements are settled in step 15 against the PDF.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>A27</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>A28</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>A30</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>A37</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>A44</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>alternative..other_values</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>moved right by one; alternative now empty</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>B37</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>timing..other_values</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>moved right by one; timing now empty</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>B42</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>timing..other_values</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>moved right by one; timing now empty</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>timing..other_values</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>moved right by one; timing now empty</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>timing..other_values</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>shifted one column left</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>moved right by one; timing now empty</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>annotator layout slip: quote was in other_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Frozen gold set: built from v3 by mechanical fixes only (duplicates, column placement, step numbers, ids, A38 preferred). No value, unit, basis or quote content was changed apart from removing the shared list intro from B quotes. Remaining disagreements are settled in step 15 against the PDF.</t>
         </is>
       </c>
     </row>

</xml_diff>